<commit_message>
feat(rules): R015 guardian-consent hold for students under 18
New optional template column guardian_consent_recorded (Y/N). Under-18
students without it get a REVIEW flag, and sharing or approving a
consent-based verification is held (409, held=R015) until the
institution records consent. Seed: two diploma minors without consent
(Sneha Patil has a student login and a signed record). Demos 29/29.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RtGcgzeU7Y7c1g9UvghaEw
</commit_message>
<xml_diff>
--- a/sample_data/demo_A_kaveri_upload_2026-27.xlsx
+++ b/sample_data/demo_A_kaveri_upload_2026-27.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,11 @@
           <t>apaar_pending_reason</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>guardian_consent_recorded</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -547,6 +552,11 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -607,6 +617,11 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -667,6 +682,11 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -727,6 +747,11 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -787,6 +812,11 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -843,6 +873,11 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -903,6 +938,11 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -963,6 +1003,11 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1023,6 +1068,11 @@
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1083,6 +1133,11 @@
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1143,6 +1198,11 @@
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1203,6 +1263,11 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1263,6 +1328,11 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1323,6 +1393,11 @@
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1383,6 +1458,11 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
@@ -1441,6 +1521,11 @@
       <c r="N17" t="inlineStr">
         <is>
           <t>FOREIGN_NATIONAL</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>

</xml_diff>